<commit_message>
Caminar en Secundaria abreviado como CS
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014d8MKHYBirCXEiF62MKJAz
</commit_message>
<xml_diff>
--- a/ICET_Ubicacion_Docentes_Bachillerato.xlsx
+++ b/ICET_Ubicacion_Docentes_Bachillerato.xlsx
@@ -3427,7 +3427,7 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="36" customWidth="1" min="10" max="10"/>
     <col width="36" customWidth="1" min="11" max="11"/>
-    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
     <col width="36" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="24" customWidth="1" min="15" max="15"/>
@@ -4212,7 +4212,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -4273,7 +4273,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -4334,7 +4334,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -4395,7 +4395,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -5836,7 +5836,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M36" t="inlineStr"/>
@@ -5897,7 +5897,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M37" t="inlineStr"/>
@@ -5958,7 +5958,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
@@ -6019,7 +6019,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
@@ -7562,7 +7562,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -7627,7 +7627,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M63" t="inlineStr"/>
@@ -7688,7 +7688,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M64" t="inlineStr"/>
@@ -7749,7 +7749,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M65" t="inlineStr"/>
@@ -9146,7 +9146,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -9211,7 +9211,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M87" t="inlineStr"/>
@@ -9272,7 +9272,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M88" t="inlineStr"/>
@@ -9333,7 +9333,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M89" t="inlineStr"/>
@@ -10612,7 +10612,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M108" t="inlineStr"/>
@@ -10673,7 +10673,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M109" t="inlineStr"/>
@@ -10734,7 +10734,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M110" t="inlineStr"/>
@@ -10795,7 +10795,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M111" t="inlineStr"/>
@@ -12512,7 +12512,7 @@
       <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M136" t="inlineStr"/>
@@ -12573,7 +12573,7 @@
       <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M137" t="inlineStr"/>
@@ -12634,7 +12634,7 @@
       <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M138" t="inlineStr"/>
@@ -12695,7 +12695,7 @@
       <c r="K139" t="inlineStr"/>
       <c r="L139" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M139" t="inlineStr"/>
@@ -14603,7 +14603,7 @@
       <c r="K167" t="inlineStr"/>
       <c r="L167" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M167" t="inlineStr"/>
@@ -14664,7 +14664,7 @@
       <c r="K168" t="inlineStr"/>
       <c r="L168" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M168" t="inlineStr"/>
@@ -14725,7 +14725,7 @@
       <c r="K169" t="inlineStr"/>
       <c r="L169" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M169" t="inlineStr"/>
@@ -15086,7 +15086,7 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M174" t="inlineStr">
@@ -15159,7 +15159,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M175" t="inlineStr">
@@ -15232,7 +15232,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M176" t="inlineStr">
@@ -15305,7 +15305,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M177" t="inlineStr">
@@ -16195,7 +16195,7 @@
       <c r="K191" t="inlineStr"/>
       <c r="L191" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M191" t="inlineStr"/>
@@ -16256,7 +16256,7 @@
       <c r="K192" t="inlineStr"/>
       <c r="L192" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M192" t="inlineStr"/>
@@ -16317,7 +16317,7 @@
       <c r="K193" t="inlineStr"/>
       <c r="L193" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M193" t="inlineStr"/>
@@ -16678,7 +16678,7 @@
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M198" t="inlineStr">
@@ -16751,7 +16751,7 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
@@ -16824,7 +16824,7 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
@@ -16897,7 +16897,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">
@@ -17515,7 +17515,7 @@
       <c r="K211" t="inlineStr"/>
       <c r="L211" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M211" t="inlineStr">
@@ -17580,7 +17580,7 @@
       <c r="K212" t="inlineStr"/>
       <c r="L212" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M212" t="inlineStr"/>
@@ -18671,7 +18671,7 @@
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M227" t="inlineStr">
@@ -18744,7 +18744,7 @@
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M228" t="inlineStr">
@@ -18817,7 +18817,7 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M229" t="inlineStr">
@@ -18890,7 +18890,7 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M230" t="inlineStr">
@@ -19508,7 +19508,7 @@
       <c r="K240" t="inlineStr"/>
       <c r="L240" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M240" t="inlineStr">
@@ -19573,7 +19573,7 @@
       <c r="K241" t="inlineStr"/>
       <c r="L241" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M241" t="inlineStr"/>
@@ -20664,7 +20664,7 @@
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M256" t="inlineStr">
@@ -20737,7 +20737,7 @@
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M257" t="inlineStr">
@@ -20810,7 +20810,7 @@
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M258" t="inlineStr">
@@ -20883,7 +20883,7 @@
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M259" t="inlineStr">
@@ -21712,7 +21712,7 @@
       <c r="K272" t="inlineStr"/>
       <c r="L272" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M272" t="inlineStr"/>
@@ -21777,7 +21777,7 @@
       <c r="K273" t="inlineStr"/>
       <c r="L273" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
@@ -21846,7 +21846,7 @@
       <c r="K274" t="inlineStr"/>
       <c r="L274" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M274" t="inlineStr">
@@ -22503,7 +22503,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
@@ -22576,7 +22576,7 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
@@ -22649,7 +22649,7 @@
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M285" t="inlineStr">
@@ -22722,7 +22722,7 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M286" t="inlineStr">
@@ -23551,7 +23551,7 @@
       <c r="K299" t="inlineStr"/>
       <c r="L299" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M299" t="inlineStr"/>
@@ -23616,7 +23616,7 @@
       <c r="K300" t="inlineStr"/>
       <c r="L300" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M300" t="inlineStr">
@@ -23685,7 +23685,7 @@
       <c r="K301" t="inlineStr"/>
       <c r="L301" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M301" t="inlineStr">
@@ -24342,7 +24342,7 @@
       </c>
       <c r="L310" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M310" t="inlineStr">
@@ -24415,7 +24415,7 @@
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M311" t="inlineStr">
@@ -24488,7 +24488,7 @@
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M312" t="inlineStr">
@@ -24561,7 +24561,7 @@
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M313" t="inlineStr">
@@ -25378,7 +25378,7 @@
       <c r="K326" t="inlineStr"/>
       <c r="L326" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M326" t="inlineStr">
@@ -25443,7 +25443,7 @@
       <c r="K327" t="inlineStr"/>
       <c r="L327" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M327" t="inlineStr"/>
@@ -25504,7 +25504,7 @@
       <c r="K328" t="inlineStr"/>
       <c r="L328" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M328" t="inlineStr"/>
@@ -26011,7 +26011,7 @@
       </c>
       <c r="L335" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M335" t="inlineStr">
@@ -26084,7 +26084,7 @@
       </c>
       <c r="L336" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M336" t="inlineStr">
@@ -26157,7 +26157,7 @@
       </c>
       <c r="L337" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M337" t="inlineStr">
@@ -26230,7 +26230,7 @@
       </c>
       <c r="L338" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M338" t="inlineStr">
@@ -27047,7 +27047,7 @@
       <c r="K351" t="inlineStr"/>
       <c r="L351" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M351" t="inlineStr">
@@ -27112,7 +27112,7 @@
       <c r="K352" t="inlineStr"/>
       <c r="L352" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M352" t="inlineStr"/>
@@ -27173,7 +27173,7 @@
       <c r="K353" t="inlineStr"/>
       <c r="L353" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M353" t="inlineStr"/>
@@ -27680,7 +27680,7 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -27753,7 +27753,7 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -27826,7 +27826,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -27899,7 +27899,7 @@
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -28606,7 +28606,7 @@
       <c r="K374" t="inlineStr"/>
       <c r="L374" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M374" t="inlineStr"/>
@@ -28667,7 +28667,7 @@
       <c r="K375" t="inlineStr"/>
       <c r="L375" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M375" t="inlineStr"/>
@@ -28728,7 +28728,7 @@
       <c r="K376" t="inlineStr"/>
       <c r="L376" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M376" t="inlineStr"/>
@@ -28793,7 +28793,7 @@
       <c r="K377" t="inlineStr"/>
       <c r="L377" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M377" t="inlineStr">
@@ -30376,7 +30376,7 @@
       <c r="K400" t="inlineStr"/>
       <c r="L400" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M400" t="inlineStr"/>
@@ -30437,7 +30437,7 @@
       <c r="K401" t="inlineStr"/>
       <c r="L401" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M401" t="inlineStr"/>
@@ -30498,7 +30498,7 @@
       <c r="K402" t="inlineStr"/>
       <c r="L402" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M402" t="inlineStr"/>
@@ -30563,7 +30563,7 @@
       <c r="K403" t="inlineStr"/>
       <c r="L403" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M403" t="inlineStr">
@@ -32183,7 +32183,7 @@
       <c r="K427" t="inlineStr"/>
       <c r="L427" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M427" t="inlineStr"/>
@@ -32248,7 +32248,7 @@
       <c r="K428" t="inlineStr"/>
       <c r="L428" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M428" t="inlineStr">
@@ -32759,7 +32759,7 @@
       </c>
       <c r="L435" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M435" t="inlineStr">
@@ -32832,7 +32832,7 @@
       </c>
       <c r="L436" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M436" t="inlineStr">
@@ -32905,7 +32905,7 @@
       </c>
       <c r="L437" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M437" t="inlineStr">
@@ -32978,7 +32978,7 @@
       </c>
       <c r="L438" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M438" t="inlineStr">
@@ -33722,7 +33722,7 @@
       <c r="K450" t="inlineStr"/>
       <c r="L450" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M450" t="inlineStr"/>
@@ -33787,7 +33787,7 @@
       <c r="K451" t="inlineStr"/>
       <c r="L451" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M451" t="inlineStr">
@@ -34298,7 +34298,7 @@
       </c>
       <c r="L458" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M458" t="inlineStr">
@@ -34371,7 +34371,7 @@
       </c>
       <c r="L459" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M459" t="inlineStr">
@@ -34444,7 +34444,7 @@
       </c>
       <c r="L460" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M460" t="inlineStr">
@@ -34517,7 +34517,7 @@
       </c>
       <c r="L461" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M461" t="inlineStr">
@@ -35322,7 +35322,7 @@
       <c r="K474" t="inlineStr"/>
       <c r="L474" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M474" t="inlineStr"/>
@@ -35387,7 +35387,7 @@
       <c r="K475" t="inlineStr"/>
       <c r="L475" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M475" t="inlineStr">
@@ -35456,7 +35456,7 @@
       <c r="K476" t="inlineStr"/>
       <c r="L476" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M476" t="inlineStr">
@@ -36113,7 +36113,7 @@
       </c>
       <c r="L485" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M485" t="inlineStr">
@@ -36186,7 +36186,7 @@
       </c>
       <c r="L486" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M486" t="inlineStr">
@@ -36259,7 +36259,7 @@
       </c>
       <c r="L487" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M487" t="inlineStr">
@@ -36332,7 +36332,7 @@
       </c>
       <c r="L488" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M488" t="inlineStr">
@@ -37137,7 +37137,7 @@
       <c r="K501" t="inlineStr"/>
       <c r="L501" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M501" t="inlineStr"/>
@@ -37202,7 +37202,7 @@
       <c r="K502" t="inlineStr"/>
       <c r="L502" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M502" t="inlineStr">
@@ -37271,7 +37271,7 @@
       <c r="K503" t="inlineStr"/>
       <c r="L503" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M503" t="inlineStr">
@@ -37928,7 +37928,7 @@
       </c>
       <c r="L512" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M512" t="inlineStr">
@@ -38001,7 +38001,7 @@
       </c>
       <c r="L513" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M513" t="inlineStr">
@@ -38074,7 +38074,7 @@
       </c>
       <c r="L514" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M514" t="inlineStr">
@@ -38147,7 +38147,7 @@
       </c>
       <c r="L515" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M515" t="inlineStr">
@@ -38907,7 +38907,7 @@
       <c r="K527" t="inlineStr"/>
       <c r="L527" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M527" t="inlineStr"/>
@@ -38968,7 +38968,7 @@
       <c r="K528" t="inlineStr"/>
       <c r="L528" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M528" t="inlineStr"/>
@@ -39029,7 +39029,7 @@
       <c r="K529" t="inlineStr"/>
       <c r="L529" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M529" t="inlineStr"/>
@@ -39090,7 +39090,7 @@
       <c r="K530" t="inlineStr"/>
       <c r="L530" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M530" t="inlineStr"/>
@@ -40576,7 +40576,7 @@
       <c r="K552" t="inlineStr"/>
       <c r="L552" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M552" t="inlineStr"/>
@@ -40637,7 +40637,7 @@
       <c r="K553" t="inlineStr"/>
       <c r="L553" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M553" t="inlineStr"/>
@@ -40698,7 +40698,7 @@
       <c r="K554" t="inlineStr"/>
       <c r="L554" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M554" t="inlineStr"/>
@@ -40759,7 +40759,7 @@
       <c r="K555" t="inlineStr"/>
       <c r="L555" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M555" t="inlineStr"/>
@@ -42139,7 +42139,7 @@
       <c r="K575" t="inlineStr"/>
       <c r="L575" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M575" t="inlineStr"/>
@@ -42204,7 +42204,7 @@
       <c r="K576" t="inlineStr"/>
       <c r="L576" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M576" t="inlineStr">
@@ -42269,7 +42269,7 @@
       <c r="K577" t="inlineStr"/>
       <c r="L577" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M577" t="inlineStr"/>
@@ -42330,7 +42330,7 @@
       <c r="K578" t="inlineStr"/>
       <c r="L578" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M578" t="inlineStr"/>
@@ -44148,7 +44148,7 @@
       <c r="K604" t="inlineStr"/>
       <c r="L604" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M604" t="inlineStr"/>
@@ -44213,7 +44213,7 @@
       <c r="K605" t="inlineStr"/>
       <c r="L605" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M605" t="inlineStr">
@@ -44278,7 +44278,7 @@
       <c r="K606" t="inlineStr"/>
       <c r="L606" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M606" t="inlineStr"/>
@@ -44339,7 +44339,7 @@
       <c r="K607" t="inlineStr"/>
       <c r="L607" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M607" t="inlineStr"/>
@@ -46186,7 +46186,7 @@
       <c r="K634" t="inlineStr"/>
       <c r="L634" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M634" t="inlineStr"/>
@@ -46251,7 +46251,7 @@
       <c r="K635" t="inlineStr"/>
       <c r="L635" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M635" t="inlineStr">
@@ -47054,7 +47054,7 @@
       </c>
       <c r="L646" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M646" t="inlineStr">
@@ -47127,7 +47127,7 @@
       </c>
       <c r="L647" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M647" t="inlineStr">
@@ -47200,7 +47200,7 @@
       </c>
       <c r="L648" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M648" t="inlineStr">
@@ -47273,7 +47273,7 @@
       </c>
       <c r="L649" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M649" t="inlineStr">
@@ -47956,7 +47956,7 @@
       <c r="K660" t="inlineStr"/>
       <c r="L660" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M660" t="inlineStr"/>
@@ -48021,7 +48021,7 @@
       <c r="K661" t="inlineStr"/>
       <c r="L661" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M661" t="inlineStr">
@@ -48824,7 +48824,7 @@
       </c>
       <c r="L672" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M672" t="inlineStr">
@@ -48897,7 +48897,7 @@
       </c>
       <c r="L673" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M673" t="inlineStr">
@@ -48970,7 +48970,7 @@
       </c>
       <c r="L674" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M674" t="inlineStr">
@@ -49043,7 +49043,7 @@
       </c>
       <c r="L675" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M675" t="inlineStr">
@@ -49941,7 +49941,7 @@
       <c r="K689" t="inlineStr"/>
       <c r="L689" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M689" t="inlineStr"/>
@@ -50002,7 +50002,7 @@
       <c r="K690" t="inlineStr"/>
       <c r="L690" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M690" t="inlineStr"/>
@@ -50067,7 +50067,7 @@
       <c r="K691" t="inlineStr"/>
       <c r="L691" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M691" t="inlineStr">
@@ -50132,7 +50132,7 @@
       <c r="K692" t="inlineStr"/>
       <c r="L692" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M692" t="inlineStr"/>
@@ -51318,7 +51318,7 @@
       <c r="K710" t="inlineStr"/>
       <c r="L710" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M710" t="inlineStr"/>
@@ -51379,7 +51379,7 @@
       <c r="K711" t="inlineStr"/>
       <c r="L711" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M711" t="inlineStr"/>
@@ -51444,7 +51444,7 @@
       <c r="K712" t="inlineStr"/>
       <c r="L712" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M712" t="inlineStr">
@@ -51509,7 +51509,7 @@
       <c r="K713" t="inlineStr"/>
       <c r="L713" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M713" t="inlineStr"/>
@@ -52549,7 +52549,7 @@
       <c r="K729" t="inlineStr"/>
       <c r="L729" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M729" t="inlineStr"/>
@@ -52610,7 +52610,7 @@
       <c r="K730" t="inlineStr"/>
       <c r="L730" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M730" t="inlineStr"/>
@@ -52675,7 +52675,7 @@
       <c r="K731" t="inlineStr"/>
       <c r="L731" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M731" t="inlineStr">
@@ -53478,7 +53478,7 @@
       </c>
       <c r="L742" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M742" t="inlineStr">
@@ -53551,7 +53551,7 @@
       </c>
       <c r="L743" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M743" t="inlineStr">
@@ -53624,7 +53624,7 @@
       </c>
       <c r="L744" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M744" t="inlineStr">
@@ -53697,7 +53697,7 @@
       </c>
       <c r="L745" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M745" t="inlineStr">
@@ -54449,7 +54449,7 @@
       <c r="K757" t="inlineStr"/>
       <c r="L757" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M757" t="inlineStr"/>
@@ -54510,7 +54510,7 @@
       <c r="K758" t="inlineStr"/>
       <c r="L758" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M758" t="inlineStr"/>
@@ -54575,7 +54575,7 @@
       <c r="K759" t="inlineStr"/>
       <c r="L759" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M759" t="inlineStr">
@@ -55378,7 +55378,7 @@
       </c>
       <c r="L770" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M770" t="inlineStr">
@@ -55451,7 +55451,7 @@
       </c>
       <c r="L771" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M771" t="inlineStr">
@@ -55524,7 +55524,7 @@
       </c>
       <c r="L772" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M772" t="inlineStr">
@@ -55597,7 +55597,7 @@
       </c>
       <c r="L773" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M773" t="inlineStr">
@@ -56361,7 +56361,7 @@
       <c r="K785" t="inlineStr"/>
       <c r="L785" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M785" t="inlineStr">
@@ -56426,7 +56426,7 @@
       <c r="K786" t="inlineStr"/>
       <c r="L786" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M786" t="inlineStr"/>
@@ -56487,7 +56487,7 @@
       <c r="K787" t="inlineStr"/>
       <c r="L787" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M787" t="inlineStr"/>
@@ -57140,7 +57140,7 @@
       </c>
       <c r="L796" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M796" t="inlineStr">
@@ -57213,7 +57213,7 @@
       </c>
       <c r="L797" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M797" t="inlineStr">
@@ -57286,7 +57286,7 @@
       </c>
       <c r="L798" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M798" t="inlineStr">
@@ -57359,7 +57359,7 @@
       </c>
       <c r="L799" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M799" t="inlineStr">
@@ -58123,7 +58123,7 @@
       <c r="K811" t="inlineStr"/>
       <c r="L811" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M811" t="inlineStr">
@@ -58188,7 +58188,7 @@
       <c r="K812" t="inlineStr"/>
       <c r="L812" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M812" t="inlineStr"/>
@@ -58249,7 +58249,7 @@
       <c r="K813" t="inlineStr"/>
       <c r="L813" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M813" t="inlineStr"/>
@@ -58902,7 +58902,7 @@
       </c>
       <c r="L822" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M822" t="inlineStr">
@@ -58975,7 +58975,7 @@
       </c>
       <c r="L823" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M823" t="inlineStr">
@@ -59048,7 +59048,7 @@
       </c>
       <c r="L824" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M824" t="inlineStr">
@@ -59121,7 +59121,7 @@
       </c>
       <c r="L825" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M825" t="inlineStr">
@@ -60003,7 +60003,7 @@
       <c r="K839" t="inlineStr"/>
       <c r="L839" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M839" t="inlineStr"/>
@@ -60364,7 +60364,7 @@
       </c>
       <c r="L844" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M844" t="inlineStr">
@@ -60437,7 +60437,7 @@
       </c>
       <c r="L845" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M845" t="inlineStr">
@@ -60510,7 +60510,7 @@
       </c>
       <c r="L846" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M846" t="inlineStr">
@@ -60583,7 +60583,7 @@
       </c>
       <c r="L847" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M847" t="inlineStr">
@@ -60656,7 +60656,7 @@
       </c>
       <c r="L848" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M848" t="inlineStr">
@@ -60729,7 +60729,7 @@
       </c>
       <c r="L849" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M849" t="inlineStr">
@@ -60802,7 +60802,7 @@
       </c>
       <c r="L850" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M850" t="inlineStr">
@@ -60875,7 +60875,7 @@
       </c>
       <c r="L851" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M851" t="inlineStr">
@@ -61757,7 +61757,7 @@
       <c r="K865" t="inlineStr"/>
       <c r="L865" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M865" t="inlineStr"/>
@@ -62118,7 +62118,7 @@
       </c>
       <c r="L870" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M870" t="inlineStr">
@@ -62191,7 +62191,7 @@
       </c>
       <c r="L871" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-1</t>
+          <t>ÉNFASIS CS 1-1</t>
         </is>
       </c>
       <c r="M871" t="inlineStr">
@@ -62264,7 +62264,7 @@
       </c>
       <c r="L872" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M872" t="inlineStr">
@@ -62337,7 +62337,7 @@
       </c>
       <c r="L873" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 1-2</t>
+          <t>ÉNFASIS CS 1-2</t>
         </is>
       </c>
       <c r="M873" t="inlineStr">
@@ -62410,7 +62410,7 @@
       </c>
       <c r="L874" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M874" t="inlineStr">
@@ -62483,7 +62483,7 @@
       </c>
       <c r="L875" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M875" t="inlineStr">
@@ -62556,7 +62556,7 @@
       </c>
       <c r="L876" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M876" t="inlineStr">
@@ -62629,7 +62629,7 @@
       </c>
       <c r="L877" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-1</t>
+          <t>ÉNFASIS CS 2-1</t>
         </is>
       </c>
       <c r="M877" t="inlineStr">
@@ -63369,7 +63369,7 @@
       <c r="K889" t="inlineStr"/>
       <c r="L889" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M889" t="inlineStr">
@@ -63438,7 +63438,7 @@
       <c r="K890" t="inlineStr"/>
       <c r="L890" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M890" t="inlineStr">
@@ -63503,7 +63503,7 @@
       <c r="K891" t="inlineStr"/>
       <c r="L891" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M891" t="inlineStr"/>
@@ -63564,7 +63564,7 @@
       <c r="K892" t="inlineStr"/>
       <c r="L892" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M892" t="inlineStr"/>
@@ -65176,7 +65176,7 @@
       <c r="K916" t="inlineStr"/>
       <c r="L916" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M916" t="inlineStr">
@@ -65245,7 +65245,7 @@
       <c r="K917" t="inlineStr"/>
       <c r="L917" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M917" t="inlineStr">
@@ -65310,7 +65310,7 @@
       <c r="K918" t="inlineStr"/>
       <c r="L918" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M918" t="inlineStr"/>
@@ -65371,7 +65371,7 @@
       <c r="K919" t="inlineStr"/>
       <c r="L919" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M919" t="inlineStr"/>
@@ -67072,7 +67072,7 @@
       <c r="K944" t="inlineStr"/>
       <c r="L944" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M944" t="inlineStr"/>
@@ -67133,7 +67133,7 @@
       <c r="K945" t="inlineStr"/>
       <c r="L945" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M945" t="inlineStr"/>
@@ -67194,7 +67194,7 @@
       <c r="K946" t="inlineStr"/>
       <c r="L946" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M946" t="inlineStr"/>
@@ -67847,7 +67847,7 @@
       </c>
       <c r="L955" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M955" t="inlineStr">
@@ -67920,7 +67920,7 @@
       </c>
       <c r="L956" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M956" t="inlineStr">
@@ -67993,7 +67993,7 @@
       </c>
       <c r="L957" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M957" t="inlineStr">
@@ -68066,7 +68066,7 @@
       </c>
       <c r="L958" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M958" t="inlineStr">
@@ -68895,7 +68895,7 @@
       <c r="K971" t="inlineStr"/>
       <c r="L971" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M971" t="inlineStr"/>
@@ -68956,7 +68956,7 @@
       <c r="K972" t="inlineStr"/>
       <c r="L972" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M972" t="inlineStr"/>
@@ -69017,7 +69017,7 @@
       <c r="K973" t="inlineStr"/>
       <c r="L973" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M973" t="inlineStr"/>
@@ -69670,7 +69670,7 @@
       </c>
       <c r="L982" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M982" t="inlineStr">
@@ -69743,7 +69743,7 @@
       </c>
       <c r="L983" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M983" t="inlineStr">
@@ -69816,7 +69816,7 @@
       </c>
       <c r="L984" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M984" t="inlineStr">
@@ -69889,7 +69889,7 @@
       </c>
       <c r="L985" t="inlineStr">
         <is>
-          <t>ÉNFASIS Caminar en Secundaria 2-2</t>
+          <t>ÉNFASIS CS 2-2</t>
         </is>
       </c>
       <c r="M985" t="inlineStr">
@@ -70718,7 +70718,7 @@
       <c r="K998" t="inlineStr"/>
       <c r="L998" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M998" t="inlineStr"/>
@@ -70779,7 +70779,7 @@
       <c r="K999" t="inlineStr"/>
       <c r="L999" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M999" t="inlineStr"/>
@@ -70840,7 +70840,7 @@
       <c r="K1000" t="inlineStr"/>
       <c r="L1000" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M1000" t="inlineStr"/>
@@ -70901,7 +70901,7 @@
       <c r="K1001" t="inlineStr"/>
       <c r="L1001" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M1001" t="inlineStr"/>
@@ -72018,7 +72018,7 @@
       <c r="K1018" t="inlineStr"/>
       <c r="L1018" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="M1018" t="inlineStr"/>
@@ -72079,7 +72079,7 @@
       <c r="K1019" t="inlineStr"/>
       <c r="L1019" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="M1019" t="inlineStr"/>
@@ -72140,7 +72140,7 @@
       <c r="K1020" t="inlineStr"/>
       <c r="L1020" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="M1020" t="inlineStr"/>
@@ -72201,7 +72201,7 @@
       <c r="K1021" t="inlineStr"/>
       <c r="L1021" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="M1021" t="inlineStr"/>
@@ -72776,7 +72776,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -72831,7 +72831,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-1</t>
+          <t>CS 1-1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -72844,7 +72844,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 1-2</t>
+          <t>CS 1-2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -72961,7 +72961,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-1</t>
+          <t>CS 2-1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -72974,7 +72974,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Caminar en Secundaria 2-2</t>
+          <t>CS 2-2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>

</xml_diff>

<commit_message>
Educación Física: intercambio de Docente 1 y 2 (datos, libros y herramienta de corrección del libro en uso), versión 2026.10.20-k
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014d8MKHYBirCXEiF62MKJAz
</commit_message>
<xml_diff>
--- a/ICET_Ubicacion_Docentes_Bachillerato.xlsx
+++ b/ICET_Ubicacion_Docentes_Bachillerato.xlsx
@@ -4637,11 +4637,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -6261,11 +6261,11 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -6955,11 +6955,11 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -7589,11 +7589,11 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -8539,11 +8539,11 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -9173,11 +9173,11 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -9940,11 +9940,11 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -10192,11 +10192,11 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -11840,11 +11840,11 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -12092,11 +12092,11 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -14565,11 +14565,11 @@
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -16157,11 +16157,11 @@
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -17046,11 +17046,11 @@
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -19039,11 +19039,11 @@
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -25405,11 +25405,11 @@
     </row>
     <row r="327">
       <c r="A327" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -27074,11 +27074,11 @@
     </row>
     <row r="352">
       <c r="A352" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -29039,11 +29039,11 @@
     </row>
     <row r="381">
       <c r="A381" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -30809,11 +30809,11 @@
     </row>
     <row r="407">
       <c r="A407" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -31527,11 +31527,11 @@
     </row>
     <row r="417">
       <c r="A417" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -33066,11 +33066,11 @@
     </row>
     <row r="440">
       <c r="A440" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -34849,11 +34849,11 @@
     </row>
     <row r="467">
       <c r="A467" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
@@ -36664,11 +36664,11 @@
     </row>
     <row r="494">
       <c r="A494" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
@@ -38442,11 +38442,11 @@
     </row>
     <row r="520">
       <c r="A520" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
@@ -38869,11 +38869,11 @@
     </row>
     <row r="527">
       <c r="A527" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
@@ -40111,11 +40111,11 @@
     </row>
     <row r="545">
       <c r="A545" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C545" t="inlineStr">
@@ -40538,11 +40538,11 @@
     </row>
     <row r="552">
       <c r="A552" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C552" t="inlineStr">
@@ -42572,11 +42572,11 @@
     </row>
     <row r="582">
       <c r="A582" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C582" t="inlineStr">
@@ -44581,11 +44581,11 @@
     </row>
     <row r="611">
       <c r="A611" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
@@ -46497,11 +46497,11 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
@@ -48267,11 +48267,11 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
@@ -49070,11 +49070,11 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C676" t="inlineStr">
@@ -49200,11 +49200,11 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C678" t="inlineStr">
@@ -50447,11 +50447,11 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C697" t="inlineStr">
@@ -50577,11 +50577,11 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C699" t="inlineStr">
@@ -52015,11 +52015,11 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
@@ -53915,11 +53915,11 @@
     </row>
     <row r="749">
       <c r="A749" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C749" t="inlineStr">
@@ -56729,11 +56729,11 @@
     </row>
     <row r="791">
       <c r="A791" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B791" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C791" t="inlineStr">
@@ -58491,11 +58491,11 @@
     </row>
     <row r="817">
       <c r="A817" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B817" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C817" t="inlineStr">
@@ -59270,11 +59270,11 @@
     </row>
     <row r="828">
       <c r="A828" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C828" t="inlineStr">
@@ -61024,11 +61024,11 @@
     </row>
     <row r="854">
       <c r="A854" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B854" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C854" t="inlineStr">
@@ -66339,11 +66339,11 @@
     </row>
     <row r="933">
       <c r="A933" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B933" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C933" t="inlineStr">
@@ -68162,11 +68162,11 @@
     </row>
     <row r="960">
       <c r="A960" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B960" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C960" t="inlineStr">
@@ -71143,11 +71143,11 @@
     </row>
     <row r="1005">
       <c r="A1005" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B1005" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C1005" t="inlineStr">
@@ -72443,11 +72443,11 @@
     </row>
     <row r="1025">
       <c r="A1025" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B1025" t="inlineStr">
         <is>
-          <t>Armero Dájome Jesús</t>
+          <t>Arizala Castro Roberto Carlos</t>
         </is>
       </c>
       <c r="C1025" t="inlineStr">

</xml_diff>

<commit_message>
Educación Física: intercambio completo de Docente 1 y 2 (incluye Ciencias Naturales), confirmado
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014d8MKHYBirCXEiF62MKJAz
</commit_message>
<xml_diff>
--- a/ICET_Ubicacion_Docentes_Bachillerato.xlsx
+++ b/ICET_Ubicacion_Docentes_Bachillerato.xlsx
@@ -28629,11 +28629,11 @@
     </row>
     <row r="375">
       <c r="A375" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -30399,11 +30399,11 @@
     </row>
     <row r="401">
       <c r="A401" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -35284,11 +35284,11 @@
     </row>
     <row r="474">
       <c r="A474" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
@@ -37099,11 +37099,11 @@
     </row>
     <row r="501">
       <c r="A501" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
@@ -52572,11 +52572,11 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
@@ -54472,11 +54472,11 @@
     </row>
     <row r="758">
       <c r="A758" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C758" t="inlineStr">
@@ -70680,11 +70680,11 @@
     </row>
     <row r="998">
       <c r="A998" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B998" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C998" t="inlineStr">
@@ -71980,11 +71980,11 @@
     </row>
     <row r="1018">
       <c r="A1018" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="B1018" t="inlineStr">
         <is>
-          <t>Arizala Castro Roberto Carlos</t>
+          <t>Armero Dájome Jesús</t>
         </is>
       </c>
       <c r="C1018" t="inlineStr">

</xml_diff>